<commit_message>
Add Stage D HTML evidence packages
</commit_message>
<xml_diff>
--- a/cases/stage_d/reviewer_A/stage_d_review.xlsx
+++ b/cases/stage_d/reviewer_A/stage_d_review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rf543ff042ce349e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R267e1d8d1add44f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Re0da2772ed3f42d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R130a370aa47540d9"/>
   </x:sheets>
   <x:calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </x:workbook>
@@ -815,6 +815,7 @@
         <x:v>CASE_26F615E94B29</x:v>
       </x:c>
       <x:c r="B2" s="64" t="str">
+        <x:f>HYPERLINK("cases/CASE_26F615E94B29.html","cases/stage_d/reviewer_A/cases/CASE_26F615E94B29.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_26F615E94B29.json</x:v>
       </x:c>
       <x:c r="C2" s="64" t="str">
@@ -842,6 +843,7 @@
         <x:v>CASE_1C3B62857D19</x:v>
       </x:c>
       <x:c r="B3" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_1C3B62857D19.html","cases/stage_d/reviewer_A/cases/CASE_1C3B62857D19.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_1C3B62857D19.json</x:v>
       </x:c>
       <x:c r="C3" s="65" t="str">
@@ -869,6 +871,7 @@
         <x:v>CASE_8A756AAC10B8</x:v>
       </x:c>
       <x:c r="B4" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_8A756AAC10B8.html","cases/stage_d/reviewer_A/cases/CASE_8A756AAC10B8.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_8A756AAC10B8.json</x:v>
       </x:c>
       <x:c r="C4" s="65" t="str">
@@ -896,6 +899,7 @@
         <x:v>CASE_7351FB1ECD56</x:v>
       </x:c>
       <x:c r="B5" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_7351FB1ECD56.html","cases/stage_d/reviewer_A/cases/CASE_7351FB1ECD56.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_7351FB1ECD56.json</x:v>
       </x:c>
       <x:c r="C5" s="65" t="str">
@@ -923,6 +927,7 @@
         <x:v>CASE_50556C8D545F</x:v>
       </x:c>
       <x:c r="B6" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_50556C8D545F.html","cases/stage_d/reviewer_A/cases/CASE_50556C8D545F.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_50556C8D545F.json</x:v>
       </x:c>
       <x:c r="C6" s="65" t="str">
@@ -950,6 +955,7 @@
         <x:v>CASE_9E4D3DF1CDB9</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_9E4D3DF1CDB9.html","cases/stage_d/reviewer_A/cases/CASE_9E4D3DF1CDB9.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_9E4D3DF1CDB9.json</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
@@ -977,6 +983,7 @@
         <x:v>CASE_978B83E2DF72</x:v>
       </x:c>
       <x:c r="B8" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_978B83E2DF72.html","cases/stage_d/reviewer_A/cases/CASE_978B83E2DF72.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_978B83E2DF72.json</x:v>
       </x:c>
       <x:c r="C8" s="65" t="str">
@@ -1004,6 +1011,7 @@
         <x:v>CASE_188C69620856</x:v>
       </x:c>
       <x:c r="B9" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_188C69620856.html","cases/stage_d/reviewer_A/cases/CASE_188C69620856.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_188C69620856.json</x:v>
       </x:c>
       <x:c r="C9" s="65" t="str">
@@ -1031,6 +1039,7 @@
         <x:v>CASE_EE7F13CD9FB7</x:v>
       </x:c>
       <x:c r="B10" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_EE7F13CD9FB7.html","cases/stage_d/reviewer_A/cases/CASE_EE7F13CD9FB7.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_EE7F13CD9FB7.json</x:v>
       </x:c>
       <x:c r="C10" s="65" t="str">
@@ -1058,6 +1067,7 @@
         <x:v>CASE_AD8C4F13A90B</x:v>
       </x:c>
       <x:c r="B11" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_AD8C4F13A90B.html","cases/stage_d/reviewer_A/cases/CASE_AD8C4F13A90B.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_AD8C4F13A90B.json</x:v>
       </x:c>
       <x:c r="C11" s="65" t="str">
@@ -1085,6 +1095,7 @@
         <x:v>CASE_091B52A05DEF</x:v>
       </x:c>
       <x:c r="B12" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_091B52A05DEF.html","cases/stage_d/reviewer_A/cases/CASE_091B52A05DEF.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_091B52A05DEF.json</x:v>
       </x:c>
       <x:c r="C12" s="65" t="str">
@@ -1112,6 +1123,7 @@
         <x:v>CASE_6C65BC36BF60</x:v>
       </x:c>
       <x:c r="B13" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_6C65BC36BF60.html","cases/stage_d/reviewer_A/cases/CASE_6C65BC36BF60.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_6C65BC36BF60.json</x:v>
       </x:c>
       <x:c r="C13" s="65" t="str">
@@ -1139,6 +1151,7 @@
         <x:v>CASE_B9E914A3762C</x:v>
       </x:c>
       <x:c r="B14" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_B9E914A3762C.html","cases/stage_d/reviewer_A/cases/CASE_B9E914A3762C.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_B9E914A3762C.json</x:v>
       </x:c>
       <x:c r="C14" s="65" t="str">
@@ -1166,6 +1179,7 @@
         <x:v>CASE_A4CDC94D210B</x:v>
       </x:c>
       <x:c r="B15" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_A4CDC94D210B.html","cases/stage_d/reviewer_A/cases/CASE_A4CDC94D210B.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_A4CDC94D210B.json</x:v>
       </x:c>
       <x:c r="C15" s="65" t="str">
@@ -1193,6 +1207,7 @@
         <x:v>CASE_5C203B1DBF11</x:v>
       </x:c>
       <x:c r="B16" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_5C203B1DBF11.html","cases/stage_d/reviewer_A/cases/CASE_5C203B1DBF11.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_5C203B1DBF11.json</x:v>
       </x:c>
       <x:c r="C16" s="65" t="str">
@@ -1220,6 +1235,7 @@
         <x:v>CASE_1FEA1F5DE7C1</x:v>
       </x:c>
       <x:c r="B17" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_1FEA1F5DE7C1.html","cases/stage_d/reviewer_A/cases/CASE_1FEA1F5DE7C1.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_1FEA1F5DE7C1.json</x:v>
       </x:c>
       <x:c r="C17" s="65" t="str">
@@ -1247,6 +1263,7 @@
         <x:v>CASE_522F0F296F37</x:v>
       </x:c>
       <x:c r="B18" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_522F0F296F37.html","cases/stage_d/reviewer_A/cases/CASE_522F0F296F37.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_522F0F296F37.json</x:v>
       </x:c>
       <x:c r="C18" s="65" t="str">
@@ -1274,6 +1291,7 @@
         <x:v>CASE_AADA2C787EEE</x:v>
       </x:c>
       <x:c r="B19" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_AADA2C787EEE.html","cases/stage_d/reviewer_A/cases/CASE_AADA2C787EEE.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_AADA2C787EEE.json</x:v>
       </x:c>
       <x:c r="C19" s="65" t="str">
@@ -1301,6 +1319,7 @@
         <x:v>CASE_5D45BE40E95A</x:v>
       </x:c>
       <x:c r="B20" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_5D45BE40E95A.html","cases/stage_d/reviewer_A/cases/CASE_5D45BE40E95A.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_5D45BE40E95A.json</x:v>
       </x:c>
       <x:c r="C20" s="65" t="str">
@@ -1328,6 +1347,7 @@
         <x:v>CASE_3A639B473AED</x:v>
       </x:c>
       <x:c r="B21" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_3A639B473AED.html","cases/stage_d/reviewer_A/cases/CASE_3A639B473AED.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_3A639B473AED.json</x:v>
       </x:c>
       <x:c r="C21" s="65" t="str">
@@ -1355,6 +1375,7 @@
         <x:v>CASE_F13F98792012</x:v>
       </x:c>
       <x:c r="B22" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_F13F98792012.html","cases/stage_d/reviewer_A/cases/CASE_F13F98792012.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_F13F98792012.json</x:v>
       </x:c>
       <x:c r="C22" s="65" t="str">
@@ -1382,6 +1403,7 @@
         <x:v>CASE_194F3A461B65</x:v>
       </x:c>
       <x:c r="B23" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_194F3A461B65.html","cases/stage_d/reviewer_A/cases/CASE_194F3A461B65.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_194F3A461B65.json</x:v>
       </x:c>
       <x:c r="C23" s="65" t="str">
@@ -1409,6 +1431,7 @@
         <x:v>CASE_C95F69523646</x:v>
       </x:c>
       <x:c r="B24" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_C95F69523646.html","cases/stage_d/reviewer_A/cases/CASE_C95F69523646.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_C95F69523646.json</x:v>
       </x:c>
       <x:c r="C24" s="65" t="str">
@@ -1436,6 +1459,7 @@
         <x:v>CASE_A1DC1299D73A</x:v>
       </x:c>
       <x:c r="B25" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_A1DC1299D73A.html","cases/stage_d/reviewer_A/cases/CASE_A1DC1299D73A.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_A1DC1299D73A.json</x:v>
       </x:c>
       <x:c r="C25" s="65" t="str">
@@ -1463,6 +1487,7 @@
         <x:v>CASE_6C2918844CE5</x:v>
       </x:c>
       <x:c r="B26" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_6C2918844CE5.html","cases/stage_d/reviewer_A/cases/CASE_6C2918844CE5.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_6C2918844CE5.json</x:v>
       </x:c>
       <x:c r="C26" s="65" t="str">
@@ -1490,6 +1515,7 @@
         <x:v>CASE_CDFEF66FCEAA</x:v>
       </x:c>
       <x:c r="B27" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_CDFEF66FCEAA.html","cases/stage_d/reviewer_A/cases/CASE_CDFEF66FCEAA.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_CDFEF66FCEAA.json</x:v>
       </x:c>
       <x:c r="C27" s="65" t="str">
@@ -1517,6 +1543,7 @@
         <x:v>CASE_DBFC2CC31FE4</x:v>
       </x:c>
       <x:c r="B28" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_DBFC2CC31FE4.html","cases/stage_d/reviewer_A/cases/CASE_DBFC2CC31FE4.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_DBFC2CC31FE4.json</x:v>
       </x:c>
       <x:c r="C28" s="65" t="str">
@@ -1544,6 +1571,7 @@
         <x:v>CASE_E6ADDBF1751F</x:v>
       </x:c>
       <x:c r="B29" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_E6ADDBF1751F.html","cases/stage_d/reviewer_A/cases/CASE_E6ADDBF1751F.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_E6ADDBF1751F.json</x:v>
       </x:c>
       <x:c r="C29" s="65" t="str">
@@ -1571,6 +1599,7 @@
         <x:v>CASE_3E3A525883BA</x:v>
       </x:c>
       <x:c r="B30" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_3E3A525883BA.html","cases/stage_d/reviewer_A/cases/CASE_3E3A525883BA.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_3E3A525883BA.json</x:v>
       </x:c>
       <x:c r="C30" s="65" t="str">
@@ -1598,6 +1627,7 @@
         <x:v>CASE_0ECE0C32A4BB</x:v>
       </x:c>
       <x:c r="B31" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_0ECE0C32A4BB.html","cases/stage_d/reviewer_A/cases/CASE_0ECE0C32A4BB.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_0ECE0C32A4BB.json</x:v>
       </x:c>
       <x:c r="C31" s="65" t="str">
@@ -1625,6 +1655,7 @@
         <x:v>CASE_34D14D6B0BB7</x:v>
       </x:c>
       <x:c r="B32" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_34D14D6B0BB7.html","cases/stage_d/reviewer_A/cases/CASE_34D14D6B0BB7.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_34D14D6B0BB7.json</x:v>
       </x:c>
       <x:c r="C32" s="65" t="str">
@@ -1652,6 +1683,7 @@
         <x:v>CASE_5FC257622E18</x:v>
       </x:c>
       <x:c r="B33" s="65" t="str">
+        <x:f>HYPERLINK("cases/CASE_5FC257622E18.html","cases/stage_d/reviewer_A/cases/CASE_5FC257622E18.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_5FC257622E18.json</x:v>
       </x:c>
       <x:c r="C33" s="65" t="str">
@@ -1679,6 +1711,7 @@
         <x:v>CASE_A0301CC135FC</x:v>
       </x:c>
       <x:c r="B34" s="66" t="str">
+        <x:f>HYPERLINK("cases/CASE_A0301CC135FC.html","cases/stage_d/reviewer_A/cases/CASE_A0301CC135FC.json")</x:f>
         <x:v>cases/stage_d/reviewer_A/cases/CASE_A0301CC135FC.json</x:v>
       </x:c>
       <x:c r="C34" s="66" t="str">

</xml_diff>